<commit_message>
added schematic for the current source
</commit_message>
<xml_diff>
--- a/bjt/currentSource.xlsx
+++ b/bjt/currentSource.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\quent\Documents\recherche\analogDesignTools\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\quent\Documents\recherche\analogDesignTools\bjt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{981D9C0B-DFCC-4D33-99A3-E15ADCF2EAD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{521CA5B6-8C06-43DE-BAD4-F32FD67FE29A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{A3A32E00-4E45-4D00-B99B-A54F1C1BA53C}"/>
   </bookViews>
@@ -36,18 +36,38 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Current source calculator for BJT</t>
   </si>
   <si>
     <t>v1.0</t>
+  </si>
+  <si>
+    <t>inputs</t>
+  </si>
+  <si>
+    <t>outputs</t>
+  </si>
+  <si>
+    <t>Vc</t>
+  </si>
+  <si>
+    <t>I@Vc</t>
+  </si>
+  <si>
+    <t>Rs+Rgnd</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="3">
+    <numFmt numFmtId="166" formatCode="0.00&quot;V&quot;"/>
+    <numFmt numFmtId="167" formatCode="0.00&quot;kΩ&quot;"/>
+    <numFmt numFmtId="168" formatCode="0.00&quot;mA&quot;"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -102,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -111,6 +131,12 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -126,6 +152,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>14289</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>642937</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>100081</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E36652E6-5697-E4FC-1BDC-F870E0547F66}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="685800" y="681039"/>
+          <a:ext cx="2547937" cy="2933767"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -445,27 +520,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{489B8EFB-5B8E-4513-8868-190D4BAA53A1}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="13.15" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="16384" width="9.06640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
+      <c r="H1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="4"/>
+      <c r="L1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="M1" s="4"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -473,11 +560,39 @@
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
     </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="H4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="I4" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="H5" t="s">
+        <v>5</v>
+      </c>
+      <c r="I5" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="H7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I7" s="6">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="A1:D2"/>
     <mergeCell ref="A3:D3"/>
+    <mergeCell ref="H1:I2"/>
+    <mergeCell ref="L1:M2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
change in conventions for clarity
</commit_message>
<xml_diff>
--- a/bjt/currentSource.xlsx
+++ b/bjt/currentSource.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\quent\Documents\recherche\analogDesignTools\bjt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{521CA5B6-8C06-43DE-BAD4-F32FD67FE29A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{625F920B-E06E-41B1-AB9F-F23F0789BE7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{A3A32E00-4E45-4D00-B99B-A54F1C1BA53C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Current source calculator for BJT</t>
   </si>
@@ -53,20 +53,43 @@
     <t>Vc</t>
   </si>
   <si>
-    <t>I@Vc</t>
-  </si>
-  <si>
-    <t>Rs+Rgnd</t>
+    <t>I(Vc)</t>
+  </si>
+  <si>
+    <t>R_S+R_GND</t>
+  </si>
+  <si>
+    <t>check</t>
+  </si>
+  <si>
+    <t>R_S</t>
+  </si>
+  <si>
+    <t>R_GND</t>
+  </si>
+  <si>
+    <t>β</t>
+  </si>
+  <si>
+    <t>V cutoff</t>
+  </si>
+  <si>
+    <t>slope</t>
+  </si>
+  <si>
+    <t>R_E</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
-    <numFmt numFmtId="166" formatCode="0.00&quot;V&quot;"/>
-    <numFmt numFmtId="167" formatCode="0.00&quot;kΩ&quot;"/>
-    <numFmt numFmtId="168" formatCode="0.00&quot;mA&quot;"/>
+  <numFmts count="5">
+    <numFmt numFmtId="164" formatCode="0.00&quot;V&quot;"/>
+    <numFmt numFmtId="165" formatCode="0.00&quot;kΩ&quot;"/>
+    <numFmt numFmtId="166" formatCode="0.00&quot;mA&quot;"/>
+    <numFmt numFmtId="167" formatCode="0.00&quot;mA/V&quot;"/>
+    <numFmt numFmtId="169" formatCode="0&quot;Ω&quot;"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -110,7 +133,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -118,25 +141,131 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -158,16 +287,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>61913</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>14289</xdr:rowOff>
+      <xdr:rowOff>61915</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>642937</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>583966</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>100081</xdr:rowOff>
+      <xdr:rowOff>9526</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -190,12 +319,17 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="685800" y="681039"/>
-          <a:ext cx="2547937" cy="2933767"/>
+          <a:off x="61913" y="752478"/>
+          <a:ext cx="2465153" cy="2838448"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -520,76 +654,135 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{489B8EFB-5B8E-4513-8868-190D4BAA53A1}">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr defaultRowHeight="13.15" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="16384" width="9.06640625" style="1"/>
+    <col min="1" max="7" width="9.06640625" style="1"/>
+    <col min="8" max="8" width="11.33203125" style="1" customWidth="1"/>
+    <col min="9" max="11" width="9.06640625" style="1"/>
+    <col min="12" max="12" width="11.33203125" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="9.06640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:17" ht="13.5" thickTop="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="H1" s="4" t="s">
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="7"/>
+      <c r="H1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="L1" s="4" t="s">
+      <c r="I1" s="7"/>
+      <c r="L1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="M1" s="4"/>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A3" s="3" t="s">
+      <c r="M1" s="7"/>
+      <c r="P1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q1" s="7"/>
+    </row>
+    <row r="2" spans="1:17" ht="13.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="8"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="10"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="15"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="15"/>
+      <c r="P2" s="14"/>
+      <c r="Q2" s="15"/>
+    </row>
+    <row r="3" spans="1:17" ht="13.9" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A3" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="13"/>
+    </row>
+    <row r="4" spans="1:17" ht="13.5" thickTop="1" x14ac:dyDescent="0.4">
       <c r="H4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="L4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M4" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="14.25" x14ac:dyDescent="0.45">
       <c r="H5" t="s">
         <v>5</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="4">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="L5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="M5" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="H6"/>
+      <c r="I6" s="4"/>
+      <c r="M6" s="16"/>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.4">
       <c r="H7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I7" s="1">
+        <v>400</v>
+      </c>
+      <c r="M7" s="16"/>
+    </row>
+    <row r="8" spans="1:17" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="H8"/>
+      <c r="I8" s="4"/>
+    </row>
+    <row r="9" spans="1:17" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="H9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I9" s="17">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.4">
+      <c r="H10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I7" s="6">
+      <c r="I10" s="3">
         <v>10</v>
       </c>
     </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.4">
+      <c r="L13" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.4">
+      <c r="L14" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A1:D2"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="H1:I2"/>
     <mergeCell ref="L1:M2"/>
+    <mergeCell ref="P1:Q2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>